<commit_message>
feat: implement request tracking and cross-team coordination
</commit_message>
<xml_diff>
--- a/operations/Operations_Control_System.xlsx
+++ b/operations/Operations_Control_System.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juangomezdev\Projects Portfolio\03_Operations_Control_System\operations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD86B055-41C6-40FD-8C09-B6CB56DDE6BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16A6DCE0-4EAF-4F25-8CE2-22EA26BE4E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requests" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="104">
   <si>
     <t>Request_ID</t>
   </si>
@@ -230,15 +230,9 @@
     <t>Retrieving PO-017 from ERP system</t>
   </si>
   <si>
-    <t>In Progress</t>
-  </si>
-  <si>
     <t>TSK-008</t>
   </si>
   <si>
-    <t>To inform to Sarah Collins or Fiannce team a inconsistency was identified</t>
-  </si>
-  <si>
     <t xml:space="preserve">REQ-003 </t>
   </si>
   <si>
@@ -270,6 +264,81 @@
   </si>
   <si>
     <t>Informing PO-017 and INV-017 Discrepancy</t>
+  </si>
+  <si>
+    <t>TSK-009</t>
+  </si>
+  <si>
+    <t>Next_Action</t>
+  </si>
+  <si>
+    <t>Follow_Up_Date</t>
+  </si>
+  <si>
+    <t>To receive certificate from Safety &amp; Compliance team</t>
+  </si>
+  <si>
+    <t>To receive communication about Invoice clarification from Sarah Collins</t>
+  </si>
+  <si>
+    <t>To inform to Sarah Collins or Fiannce team a inconsistency was identified in invoice INV-017</t>
+  </si>
+  <si>
+    <t>To send link meeting again to participants and make sure they have access to administrative requirements documents</t>
+  </si>
+  <si>
+    <t>ACT-009</t>
+  </si>
+  <si>
+    <t>Located the latest available PRJ-004 administrative requirements document (v2) and identified pending Finance validation of cost estimates.</t>
+  </si>
+  <si>
+    <t>Locating administrative requirements documents</t>
+  </si>
+  <si>
+    <t>Sending email meeting confirmation</t>
+  </si>
+  <si>
+    <t>Sent meeting reminder to Operations and Finance, shared the available document information, and requested confirmation of outstanding Finance requirements.</t>
+  </si>
+  <si>
+    <t>ACT-010</t>
+  </si>
+  <si>
+    <t>TSK-010</t>
+  </si>
+  <si>
+    <t>To request access to Michael Torres to Finance teams</t>
+  </si>
+  <si>
+    <t>ACT-011</t>
+  </si>
+  <si>
+    <t>Requesting Michael torres to grant access to documents to Finance team</t>
+  </si>
+  <si>
+    <t>Sent an email communicating Operations Manager requesting access to documents to Finance team</t>
+  </si>
+  <si>
+    <t>Waiting response</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACT-012 </t>
+  </si>
+  <si>
+    <t>Sent an email communicating Finance she was granted to access folder.</t>
+  </si>
+  <si>
+    <t>Closed</t>
+  </si>
+  <si>
+    <t>Communicating Sarah Collins access granted to folder</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Meeting finished</t>
   </si>
 </sst>
 </file>
@@ -309,14 +378,14 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -342,21 +411,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="22" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="22" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="22" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="22" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="22" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -637,23 +709,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="110.6640625" customWidth="1"/>
+    <col min="5" max="5" width="86.21875" customWidth="1"/>
     <col min="6" max="6" width="156.77734375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14.5546875" customWidth="1"/>
     <col min="9" max="9" width="25.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="26" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="71.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -687,8 +761,14 @@
       <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="L1" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -710,10 +790,10 @@
       <c r="G2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="H2" s="7">
+      <c r="H2" s="6">
         <v>46318</v>
       </c>
-      <c r="I2" s="7">
+      <c r="I2" s="6">
         <v>46316</v>
       </c>
       <c r="J2" s="1" t="s">
@@ -722,8 +802,14 @@
       <c r="K2" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="L2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="M2" s="13">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>33</v>
       </c>
@@ -745,20 +831,26 @@
       <c r="G3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H3" s="7">
+      <c r="H3" s="6">
         <v>46316</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="6">
         <v>46314</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>14</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+      <c r="L3" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="M3" s="12">
+        <v>46315.458333333336</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>46</v>
       </c>
@@ -780,10 +872,10 @@
       <c r="G4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="6">
         <v>46315</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="6">
         <v>46314</v>
       </c>
       <c r="J4" s="1" t="s">
@@ -791,6 +883,12 @@
       </c>
       <c r="K4" s="1" t="s">
         <v>32</v>
+      </c>
+      <c r="L4" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="M4" s="14" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -800,12 +898,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8747D367-1A8B-49AC-92D6-15BA2088813C}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="85.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="118" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.77734375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.21875" bestFit="1" customWidth="1"/>
@@ -832,163 +930,208 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="6">
+      <c r="D2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="5">
         <v>46314</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="9" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="6">
+      <c r="D3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="5">
         <v>46314</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="9" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="6">
+      <c r="D4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="5">
         <v>46315</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="9" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="9">
+      <c r="D5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="8">
         <v>46314</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="9" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="D6" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="9">
+      <c r="D6" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="8">
         <v>46314</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="9" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="9">
+      <c r="D7" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="8">
         <v>46314</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="9" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="D8" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" s="9">
+      <c r="D8" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="8">
         <v>46314</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="9" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" s="11" t="s">
+      <c r="A9" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9" s="12">
+      <c r="C9" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="13">
         <v>46314</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="9" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="10">
+        <v>46315</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="13">
+        <v>46315</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D18" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -998,13 +1141,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83279FCC-00E9-44CC-8AE4-756A6A5BDCD3}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="44.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="74" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23.21875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="190" bestFit="1" customWidth="1"/>
   </cols>
@@ -1030,163 +1173,243 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="12">
         <v>46311.40625</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="5" t="s">
+      <c r="E2" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="11" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="12">
         <v>46314.375</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="E3" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="8" t="s">
+      <c r="E3" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="11" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="12">
         <v>46314.416666666664</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="E4" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="8" t="s">
+      <c r="E4" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="11" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="12">
         <v>46314.4375</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="E5" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="8" t="s">
+      <c r="E5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="11" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="B6" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="12">
         <v>46314.447916666664</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="8" t="s">
+      <c r="E6" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="11" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B7" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7" s="12">
+        <v>46314.458333333336</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="11" t="s">
         <v>70</v>
-      </c>
-      <c r="C7" s="13">
-        <v>46314.458333333336</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C8" s="12">
+        <v>46314.465277777781</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="11" t="s">
         <v>75</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="C8" s="13">
-        <v>46314.465277777781</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" s="12">
+        <v>46314.472222222219</v>
+      </c>
+      <c r="D9" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="C9" s="13">
-        <v>46314.472222222219</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>80</v>
-      </c>
       <c r="E9" s="11" t="s">
         <v>14</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>79</v>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="12">
+        <v>46315.378472222219</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="12">
+        <v>46315.381944444445</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" s="12">
+        <v>46315.392361111109</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="12">
+        <v>46315.399305555555</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>